<commit_message>
Excel Kliniği ücretsiz dosyalar: son metinler, TAHLİL kapasitesi ve iki Başla düzeltmesi
- 43 ürün kaydının son metinleri (dosyaların Başla ve sayfa yapısından; kaynakta olmayan rakam yok)
- TAHLİL: LibreOffice gizli ara hesap sütunlu satırları kaydederken atıyordu (Veri 1085–2004 formülleri
  kayboluyordu); F–I sütunları artık kayıttan sonra XML'de gizleniyor, 2000 satırlık kapasite gerçekten var
- ANTRENMAN sloganı: dosyada haftalık hesap yok, "haftalık" çıkarıldı
- KİLER: aynı ürün adı iki kez girilemediği için "ayrı satır aç" önerisi çıkarıldı
- Ücretsiz ürün sayfasında "Doğrulama" satırı; raf üst bölüm notu Shopier durumuna göre

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FcJ9eYFL81XLJVo3qWny3N
</commit_message>
<xml_diff>
--- a/dosyalar/excel-klinigi/ExcelKlinigi_KILER_Erzak_Takibi.xlsx
+++ b/dosyalar/excel-klinigi/ExcelKlinigi_KILER_Erzak_Takibi.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">Tek tarih</t>
   </si>
   <si>
-    <t xml:space="preserve">Aynı üründen farklı tarihli paketler varsa en yakın tarihi yaz ya da ayrı satır aç.</t>
+    <t xml:space="preserve">Aynı üründen farklı tarihli paketler varsa en yakın tarihi yaz; her ürün adı bir kez girilir.</t>
   </si>
   <si>
     <t xml:space="preserve">Kapasite</t>
@@ -992,7 +992,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
         <v>11</v>
       </c>

</xml_diff>